<commit_message>
Cambios en la normalizacion
</commit_message>
<xml_diff>
--- a/Normalización.xlsx
+++ b/Normalización.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="64">
   <si>
     <t>IdProveedor</t>
   </si>
@@ -34,10 +34,16 @@
     <t>Patito S.A</t>
   </si>
   <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
     <t>IdAceptacion</t>
   </si>
   <si>
     <t>CondicionesPago</t>
+  </si>
+  <si>
+    <t>FechaAceptacion</t>
   </si>
   <si>
     <t>IdOrdenProveedor</t>
@@ -359,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -387,6 +393,9 @@
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -402,30 +411,33 @@
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="6" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -446,9 +458,6 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -653,11 +662,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:C7" displayName="AceptacionProveedor" name="AceptacionProveedor" id="2">
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:D7" displayName="AceptacionProveedor" name="AceptacionProveedor" id="2">
+  <tableColumns count="4">
     <tableColumn name="IdAceptacion" id="1"/>
     <tableColumn name="IdProveedor" id="2"/>
     <tableColumn name="CondicionesPago" id="3"/>
+    <tableColumn name="FechaAceptacion" id="4"/>
   </tableColumns>
   <tableStyleInfo name="Hoja 1-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -738,11 +748,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A30:C31" displayName="AceptacionCliente" name="AceptacionCliente" id="8">
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A30:D31" displayName="AceptacionCliente" name="AceptacionCliente" id="8">
+  <tableColumns count="4">
     <tableColumn name="IdAceptacionCliente" id="1"/>
     <tableColumn name="IdCliente" id="2"/>
     <tableColumn name="CondicionesPago" id="3"/>
+    <tableColumn name="FechaAceptacion" id="4"/>
   </tableColumns>
   <tableStyleInfo name="Hoja 1-style 8" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -969,7 +980,7 @@
     <col customWidth="1" min="1" max="1" width="20.5"/>
     <col customWidth="1" min="2" max="2" width="21.13"/>
     <col customWidth="1" min="3" max="3" width="36.25"/>
-    <col customWidth="1" min="4" max="4" width="14.88"/>
+    <col customWidth="1" min="4" max="4" width="19.63"/>
     <col customWidth="1" min="5" max="5" width="14.38"/>
     <col customWidth="1" min="6" max="6" width="13.38"/>
     <col customWidth="1" min="7" max="7" width="18.38"/>
@@ -1011,549 +1022,566 @@
       </c>
       <c r="G3" s="8"/>
     </row>
+    <row r="5">
+      <c r="G5" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="10" t="s">
+      <c r="A6" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>0</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B7" s="13">
+      <c r="A7" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B7" s="14">
         <v>1.0</v>
       </c>
       <c r="C7" s="14">
         <v>1.0</v>
       </c>
+      <c r="D7" s="15">
+        <v>45700.0</v>
+      </c>
     </row>
     <row r="9">
-      <c r="F9" s="15"/>
+      <c r="F9" s="16"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="B11" s="20">
+        <v>123.0</v>
+      </c>
+      <c r="C11" s="21">
+        <v>45700.0</v>
+      </c>
+      <c r="D11" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="E11" s="20">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="14">
+        <v>1500.0</v>
+      </c>
+      <c r="E15" s="14">
+        <v>250.0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0.0</v>
+      </c>
+      <c r="G15" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B19" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="C19" s="14">
+        <v>2000.0</v>
+      </c>
+      <c r="D19" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="G19" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B23" s="14">
+        <v>1231.0</v>
+      </c>
+      <c r="C23" s="14">
+        <v>50000.0</v>
+      </c>
+      <c r="D23" s="14">
+        <v>25000.0</v>
+      </c>
+      <c r="E23" s="24">
+        <v>45700.0</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0.0</v>
+      </c>
+      <c r="G23" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H26" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F27" s="14">
+        <v>5.02320122E8</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="H27" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="D30" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="B11" s="19">
-        <v>123.0</v>
-      </c>
-      <c r="C11" s="20">
+    </row>
+    <row r="31">
+      <c r="A31" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B31" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="C31" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="D31" s="15">
         <v>45700.0</v>
       </c>
-      <c r="D11" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="E11" s="19">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="10" t="s">
+    </row>
+    <row r="33">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="10" t="s">
+      <c r="D34" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="H34" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B35" s="14">
+        <v>5.06780876E8</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" s="14">
+        <v>8.8754324E7</v>
+      </c>
+      <c r="G35" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" s="14">
+        <v>123456.0</v>
+      </c>
+      <c r="I35" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C38" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="10" t="s">
+    </row>
+    <row r="39">
+      <c r="A39" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C39" s="23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" s="27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B43" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="C43" s="23">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E46" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="F46" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H46" s="25" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="13">
-        <v>1500.0</v>
-      </c>
-      <c r="E15" s="13">
-        <v>250.0</v>
-      </c>
-      <c r="F15" s="13">
+      <c r="I46" s="22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="14">
+        <v>10.0</v>
+      </c>
+      <c r="E47" s="14">
+        <v>1000.0</v>
+      </c>
+      <c r="F47" s="30">
+        <v>0.3</v>
+      </c>
+      <c r="G47" s="14">
         <v>0.0</v>
       </c>
-      <c r="G15" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="H47" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="I47" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="9"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="28"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D51" s="23">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B54" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="C54" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B19" s="13">
-        <v>2.0</v>
-      </c>
-      <c r="C19" s="13">
-        <v>2000.0</v>
-      </c>
-      <c r="D19" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="E19" s="13" t="s">
+      <c r="D54" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F19" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="G19" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B23" s="13">
-        <v>1231.0</v>
-      </c>
-      <c r="C23" s="13">
-        <v>50000.0</v>
-      </c>
-      <c r="D23" s="13">
-        <v>25000.0</v>
-      </c>
-      <c r="E23" s="22">
-        <v>45700.0</v>
-      </c>
-      <c r="F23" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="G23" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="F27" s="13">
-        <v>5.02320122E8</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H27" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B31" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="C31" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="21"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="21"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F34" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H34" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="I34" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B35" s="13">
-        <v>5.06780876E8</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F35" s="13">
-        <v>8.8754324E7</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="H35" s="13">
-        <v>123456.0</v>
-      </c>
-      <c r="I35" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="21"/>
-      <c r="B37" s="21"/>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-      <c r="G37" s="21"/>
-      <c r="H37" s="21"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="C38" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="21"/>
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B42" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C42" s="25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B43" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="C43" s="14">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="26"/>
-      <c r="B45" s="21"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="21"/>
-      <c r="F45" s="21"/>
-      <c r="G45" s="21"/>
-      <c r="H45" s="21"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C46" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H46" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="I46" s="11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B47" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D47" s="13">
-        <v>10.0</v>
-      </c>
-      <c r="E47" s="13">
-        <v>1000.0</v>
-      </c>
-      <c r="F47" s="28">
-        <v>0.3</v>
-      </c>
-      <c r="G47" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="H47" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="I47" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="21"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="26"/>
-      <c r="B49" s="21"/>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C50" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B51" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D51" s="14">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="27" t="s">
-        <v>60</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E54" s="29" t="s">
-        <v>61</v>
+      <c r="E54" s="12" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="12">
-        <v>1.0</v>
-      </c>
-      <c r="B55" s="13">
+      <c r="A55" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="B55" s="14">
         <v>5.0</v>
       </c>
-      <c r="C55" s="13">
+      <c r="C55" s="14">
         <v>7000.0</v>
       </c>
-      <c r="D55" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="E55" s="30">
+      <c r="D55" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="E55" s="31">
         <v>1.0</v>
       </c>
     </row>

</xml_diff>